<commit_message>
Add batch processing, Excel formatting, and .gitignore
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,32 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="メイリオ"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="メイリオ"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +58,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,122 +449,122 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ページ</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>テキスト</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>商品名</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>小計</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>月次売上レポート</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ノートPC</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>80,000</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>800,000</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>作成日: 2025年7月1日</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>マウス</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>100,000</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>担当者: 田中太郎</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>キーボード</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>5,000</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>150,000</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>部署: 営業部</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>商品名 数量 単価 小計</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ノートPC 10 80,000 800,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>マウス 50 2,000 100,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>キーボード 30 5,000 150,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>モニター 15 35,000 525,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>合計: 1,575,000円</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>モニター</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>35,000</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>525,000</t>
         </is>
       </c>
     </row>

</xml_diff>